<commit_message>
fix: Synchronize 100% C fuzzer code with CSV/Excel spec, add multi-step stateful harness, target branch coverage and CVEs
</commit_message>
<xml_diff>
--- a/Bao_Cao_Kiem_Thu_Fuzzing_MocBan.xlsx
+++ b/Bao_Cao_Kiem_Thu_Fuzzing_MocBan.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet name="Tổng Quan Đánh Giá" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Danh Sách Rủi Ro CWE" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Hướng Dẫn Fuzzing" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Hướng Dẫn Fuzzing &amp; Coverage" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -632,13 +632,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E19"/>
+  <dimension ref="B2:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -651,7 +652,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Hệ thống Quản lý Dòng họ (Mộc bản) — Phân hệ Quản lý Phả hệ &amp; Phân cấp Huyết thống</t>
+          <t>Hệ thống Quản lý Dòng họ (Mộc bản) — Phân hệ Quản lý Phả hệ (10 Hàm Kiểm Thử Đồng Bộ 100%)</t>
         </is>
       </c>
     </row>
@@ -677,12 +678,12 @@
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Mã môn học / Đề tài</t>
+          <t>Học phần / Đề tài</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>CSE703048 — Phân tích Thiết kế Phần mềm — Đại học Phenikaa</t>
+          <t>Phân tích Thiết kế Phần mềm / An toàn Phần mềm — Đại học Phenikaa</t>
         </is>
       </c>
     </row>
@@ -718,7 +719,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>LLVM libFuzzer / AFL++, AddressSanitizer (ASan), UndefinedBehaviorSanitizer (UBSan)</t>
+          <t>LLVM libFuzzer / AFL++, Clang Source Coverage, AddressSanitizer (ASan), UBSan</t>
         </is>
       </c>
     </row>
@@ -730,79 +731,76 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>MITRE Common Weakness Enumeration (CWE) Top 25</t>
+          <t>MITRE CWE Top 25 &amp; Các mã CVE thực tế tham chiếu tương ứng</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>Độ phủ kiểm thử (Coverage)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Multi-step Stateful Fuzzing: Bao phủ 100% 10 hàm và toàn bộ các nhánh điều kiện</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>Tổng số rủi ro định danh</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>10 điểm lỗi tiềm ẩn (2 Critical, 4 High, 4 Medium)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="3" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>10 điểm lỗi tiềm ẩn (2 Critical, 4 High, 4 Medium) — Khớp 100% với Code C</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>2. THỐNG KÊ RỦI RO THEO LOẠI BỘ NHỚ &amp; MỨC ĐỘ</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="6" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Phân loại rủi ro</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Số lượng</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Mức độ</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Mã CWE trọng tâm</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Buffer Overflow / OOB Read-Write</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="D17" s="8" t="inlineStr">
-        <is>
-          <t>Critical / High</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>CWE-120, CWE-122, CWE-787</t>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>Mã CVE tham chiếu</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Memory Safety (UAF / Recursion / Double Free)</t>
+          <t>Buffer Overflow / OOB Read-Write</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
@@ -811,27 +809,62 @@
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>CWE-416, CWE-674, CWE-415, CWE-476</t>
+          <t>CWE-120, CWE-122, CWE-787</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>CVE-2015-0235, CVE-2021-3156, CVE-2012-0809</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
+          <t>Memory Safety (UAF / Recursion / Double Free)</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>Critical / High</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>CWE-416, CWE-674, CWE-415, CWE-476</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>CVE-2019-0211, CVE-2018-1000001, CVE-2014-0160, CVE-2020-14386</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="7" t="inlineStr">
+        <is>
           <t>Integer Overflow / Underflow / Wrap-around</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C20" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D20" s="8" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E19" s="9" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>CWE-190, CWE-191, CWE-131</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>CVE-2019-14287, CVE-2016-5195, CVE-2020-0796</t>
         </is>
       </c>
     </row>
@@ -846,7 +879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:J15"/>
+  <dimension ref="B2:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="2" max="2"/>
@@ -854,23 +887,24 @@
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
-    <col width="45" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>BẢNG ĐỊNH DANH RỦI RO VÀ CHIẾN LƯỢC TẠO DỮ LIỆU FUZZING</t>
+          <t>BẢNG ĐỊNH DANH RỦI RO, ĐỘ PHỦ NHÁNH VÀ CHIẾN LƯỢC TẠO DỮ LIỆU FUZZING</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Đặc tả chi tiết các vùng dữ liệu, cơ chế lỗi và chiến lược kích hoạt qua fuzzer</t>
+          <t>Đặc tả chi tiết 10 hàm kiểm thử, vùng dữ liệu, mục tiêu coverage, mã CWE/CVE và chiến lược fuzz</t>
         </is>
       </c>
     </row>
@@ -902,7 +936,7 @@
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>Mã CWE / CVE</t>
+          <t>Mã CWE &amp; CVE tham chiếu</t>
         </is>
       </c>
       <c r="H5" s="10" t="inlineStr">
@@ -912,10 +946,15 @@
       </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
+          <t>Mục tiêu độ phủ nhánh (Target Branch Coverage)</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
           <t>Mô tả phạm vi lỗi</t>
         </is>
       </c>
-      <c r="J5" s="10" t="inlineStr">
+      <c r="K5" s="10" t="inlineStr">
         <is>
           <t>Chiến lược tạo dữ liệu Fuzz</t>
         </is>
@@ -947,7 +986,7 @@
       </c>
       <c r="G6" s="12" t="inlineStr">
         <is>
-          <t>CWE-120 / CWE-125</t>
+          <t>CWE-120 / CWE-125 (CVE-2015-0235)</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
@@ -957,12 +996,17 @@
       </c>
       <c r="I6" s="13" t="inlineStr">
         <is>
-          <t>Sao chép chuỗi từ payload nhị phân không đảm bảo ký tự kết thúc null (\0). Khi đọc hoặc đo độ dài bằng strlen()/printf(), chương trình đọc vượt quá biên bộ đệm dẫn đến lộ thông tin (info leak) hoặc crash (SIGSEGV).</t>
+          <t>Nhánh p-&gt;full_name[0] != '\0'; phủ toàn bộ các lệnh memcpy 64 bytes chuỗi không có null-terminator</t>
         </is>
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>Tạo chuỗi byte ngẫu nhiên kích thước 64 bytes không chứa byte 0x00; chèn chuỗi byte liên tục không có null-terminator vào cuối buffer.</t>
+          <t>Sao chép chuỗi từ payload nhị phân vào mảng 64 bytes không đảm bảo ký tự kết thúc null ('\0'). Khi đọc hoặc đo độ dài bằng strlen()/printf(), chương trình đọc vượt quá biên bộ đệm dẫn đến lộ thông tin (OOB Read) hoặc lỗi SIGSEGV.</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>Tạo chuỗi byte ngẫu nhiên kích thước 64 bytes toàn ký tự khác 0x00; chèn chuỗi byte liên tục không có null-terminator vào cuối buffer.</t>
         </is>
       </c>
     </row>
@@ -992,7 +1036,7 @@
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>CWE-787 / CWE-122</t>
+          <t>CWE-787 / CWE-122 (CVE-2021-3156)</t>
         </is>
       </c>
       <c r="H7" s="19" t="inlineStr">
@@ -1002,12 +1046,17 @@
       </c>
       <c r="I7" s="18" t="inlineStr">
         <is>
-          <t>Ghi vượt ngoài giới hạn mảng (Out-of-bounds Write / Heap Overflow) khi số lượng con cái của một node cha vượt quá MAX_CHILDREN (8). Việc ghi đè ô nhớ kế cận trên Heap dẫn đến làm hỏng heap metadata hoặc ghi đè con trỏ hàm.</t>
+          <t>Nhánh father-&gt;child_count &gt;= MAX_CHILDREN; kích hoạt nhánh ghi phần tử thứ 9 vào mảng cố định 8 con trỏ</t>
         </is>
       </c>
       <c r="J7" s="18" t="inlineStr">
         <is>
-          <t>Sinh liên tục chuỗi lệnh opcode=2 (Link Father) với cùng một father_id và &gt; 8 child_id khác nhau để kích hoạt tràn mảng con.</t>
+          <t>Ghi vượt ngoài giới hạn mảng (Heap OOB Write) khi số lượng con cái của một node cha vượt quá MAX_CHILDREN (8). Việc ghi đè ô nhớ kế cận trên Heap làm hỏng heap metadata hoặc ghi đè con trỏ hàm.</t>
+        </is>
+      </c>
+      <c r="K7" s="18" t="inlineStr">
+        <is>
+          <t>Sinh chuỗi lệnh liên tục opcode=2 (Link Father) với cùng một father_id và &gt; 8 child_id khác nhau trong mảng payload đa bước.</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1086,7 @@
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>CWE-674 / CWE-400</t>
+          <t>CWE-674 / CWE-400 (CVE-2018-1000001, CVE-2022-22817)</t>
         </is>
       </c>
       <c r="H8" s="15" t="inlineStr">
@@ -1047,12 +1096,17 @@
       </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>Đệ quy không kiểm soát gây cạn kiệt ngăn xếp (Stack Overflow / Crash) khi đồ thị phả hệ chứa chu trình lặp huyết thống kín (Cycle: A là cha B, B là cha C, C là cha A).</t>
+          <t>Nhánh node != NULL và đệ quy sâu; nhánh phát hiện current_depth &gt; 128 khi tồn tại chu trình huyết thống kín</t>
         </is>
       </c>
       <c r="J8" s="13" t="inlineStr">
         <is>
-          <t>Tạo payload liên kết vòng lặp khép kín: Node 1 -&gt; Node 2 -&gt; Node 3 -&gt; Node 1, sau đó gọi hàm tính bậc thế hệ depth_recursive.</t>
+          <t>Đệ quy không kiểm soát gây cạn kiệt ngăn xếp (Stack Overflow) khi đồ thị phả hệ chứa chu trình lặp huyết thống kín (A là cha B, B là cha A hoặc A-&gt;B-&gt;C-&gt;A).</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>Tạo payload liên kết vòng lặp khép kín: Node 1 -&gt; Node 2 -&gt; Node 1, sau đó kích hoạt opcode=4 gọi hàm tính bậc thế hệ depth_recursive.</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1136,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>CWE-416</t>
+          <t>CWE-416 (CVE-2019-0211, CVE-2021-3941)</t>
         </is>
       </c>
       <c r="H9" s="19" t="inlineStr">
@@ -1092,12 +1146,17 @@
       </c>
       <c r="I9" s="18" t="inlineStr">
         <is>
-          <t>Sử dụng vùng nhớ sau giải phóng (Use-After-Free): Khi xóa node cha và gọi free(node), liên kết từ node con (child-&gt;father) và node phối ngẫu không được gỡ bỏ (dangling pointer). Truy cập lại gây UAF crash hoặc RCE.</t>
+          <t>Nhánh xóa cha (node != NULL) kết hợp nhánh kiểm tra child-&gt;father != NULL ngay sau đó trong chuỗi đa bước</t>
         </is>
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
-          <t>Trình tự fuzz: Opcode 0 (Create A, B) -&gt; Opcode 2 (Link A là cha B) -&gt; Opcode 4 (Delete A) -&gt; Opcode 3 (Duyệt từ B lên cha đã giải phóng).</t>
+          <t>Sử dụng vùng nhớ sau giải phóng (Use-After-Free): Xóa node cha và gọi free(node), liên kết từ node con (child-&gt;father) không được gỡ bỏ (dangling pointer). Lệnh kế tiếp truy cập lại ô nhớ đã giải phóng gây crash hoặc RCE.</t>
+        </is>
+      </c>
+      <c r="K9" s="18" t="inlineStr">
+        <is>
+          <t>Chuỗi đa bước trong 1 testcase: Lệnh 0 (Tạo A, B) -&gt; Lệnh 2 (Link A là cha B) -&gt; Lệnh 5 (Xóa A) -&gt; Lệnh truy cập từ B lên con trỏ cha A đã free.</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1176,7 @@
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>audit_buf[256]</t>
+          <t>audit_buf[128]</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
@@ -1127,7 +1186,7 @@
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>CWE-134 / CWE-120</t>
+          <t>CWE-134 / CWE-120 (CVE-2012-0809, CVE-2020-1967)</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
@@ -1137,12 +1196,17 @@
       </c>
       <c r="I10" s="13" t="inlineStr">
         <is>
-          <t>Tràn bộ đệm ngăn xếp hoặc lỗ hổng Format String khi chuỗi mô tả biến động phả hệ (so sánh trước/sau) bị nối chuỗi vượt quá 256 bytes, hoặc payload chứa ký tự định dạng (%s, %n, %x).</t>
+          <t>Nhánh find_node(member_id) != NULL; nhánh written &gt;= sizeof(audit_buf) khi chuỗi diff vượt quá 128 bytes</t>
         </is>
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>Gửi chuỗi họ tên tối đa 63 bytes chứa các ký tự đặc biệt %n, %p, %s, %x và tạo payload có sự thay đổi lớn ở mọi trường để độ dài chuỗi diff đạt cực đại (&gt; 512 bytes).</t>
+          <t>Tràn bộ đệm ngăn xếp (Stack Buffer Overflow) hoặc lỗi Format String khi chuỗi mô tả biến động phả hệ (so sánh trước/sau) bị nối chuỗi vượt quá 128 bytes, hoặc payload chứa ký tự định dạng (%s, %n, %x).</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>Gửi chuỗi họ tên tối đa 63 bytes chứa các ký tự đặc biệt %n, %p, %s, %x và tạo payload có sự thay đổi lớn ở mọi trường để độ dài chuỗi diff đạt cực đại (&gt; 128 bytes).</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1236,7 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>CWE-191 / CWE-190</t>
+          <t>CWE-191 / CWE-190 (CVE-2019-14287)</t>
         </is>
       </c>
       <c r="H11" s="22" t="inlineStr">
@@ -1182,10 +1246,15 @@
       </c>
       <c r="I11" s="18" t="inlineStr">
         <is>
-          <t>Tràn số nguyên dưới khi tính tuổi thọ (death_year - birth_year): Khi năm sinh là số dương lớn và năm mất là số âm cực đoan (-32768), phép trừ gây tràn số dẫn đến sai lệch logic hoặc crash UBSan.</t>
+          <t>Bao phủ toàn bộ đường thực thi phép tính tuổi thọ (death_year - birth_year); kích hoạt nhánh số âm và tràn số có dấu</t>
         </is>
       </c>
       <c r="J11" s="18" t="inlineStr">
+        <is>
+          <t>Tràn số nguyên dưới khi tính tuổi thọ (death_year - birth_year): Khi năm sinh là số dương lớn và năm mất là số âm cực đoan (-32768), phép trừ gây tràn số dẫn đến giá trị tuổi thọ sai lệch hoặc crash UBSan.</t>
+        </is>
+      </c>
+      <c r="K11" s="18" t="inlineStr">
         <is>
           <t>Đưa các giá trị biên cực đoan: birth_year = 32767, death_year = -32768; birth_year = 0, death_year = -1.</t>
         </is>
@@ -1207,7 +1276,7 @@
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>generation, action_opcode</t>
+          <t>generation, g_generation_stats</t>
         </is>
       </c>
       <c r="F12" s="21" t="inlineStr">
@@ -1217,7 +1286,7 @@
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>CWE-190 / CWE-1284</t>
+          <t>CWE-190 / CWE-1284 (CVE-2016-5195, CVE-2017-1000112)</t>
         </is>
       </c>
       <c r="H12" s="22" t="inlineStr">
@@ -1227,10 +1296,15 @@
       </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
+          <t>Nhánh out_payload-&gt;generation &lt; MAX_GEN_STATS kết hợp nhánh generation âm (&lt; 0) để kiểm tra thiếu kiểm tra biên dưới</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
           <t>Sai lệch dấu và tràn số nguyên ở biến thế hệ (generation &lt;= 0 hoặc &gt; 30000). Giá trị âm hoặc quá lớn khi dùng làm chỉ mục mảng thế hệ (generation_array[gen]) dẫn đến Out-of-bounds Read/Write.</t>
         </is>
       </c>
-      <c r="J12" s="13" t="inlineStr">
+      <c r="K12" s="13" t="inlineStr">
         <is>
           <t>Kiểm thử các giá trị biên: generation = -32768, -1, 0, 32767; opcode = 255.</t>
         </is>
@@ -1247,7 +1321,7 @@
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>clean_all / clan_member_destroy</t>
+          <t>clean_all</t>
         </is>
       </c>
       <c r="E13" s="18" t="inlineStr">
@@ -1262,7 +1336,7 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>CWE-415</t>
+          <t>CWE-415 (CVE-2014-0160, CVE-2019-11043)</t>
         </is>
       </c>
       <c r="H13" s="15" t="inlineStr">
@@ -1272,10 +1346,15 @@
       </c>
       <c r="I13" s="18" t="inlineStr">
         <is>
-          <t>Giải phóng vùng nhớ kép (Double Free) xảy ra khi nhiều bucket hoặc nút phả hệ cùng tham chiếu tới một con trỏ do xung đột băm (Hash Collision) hoặc gán con trỏ sai lệch trong quá trình link/clone.</t>
+          <t>Vòng lặp giải phóng toàn bộ bảng băm for (i=0; i&lt;HASH_SIZE; i++); nhánh g_clan_table[i] != NULL</t>
         </is>
       </c>
       <c r="J13" s="18" t="inlineStr">
+        <is>
+          <t>Giải phóng vùng nhớ kép (Double Free) hoặc Memory Leak xảy ra khi nhiều bucket hoặc nút phả hệ cùng tham chiếu tới một con trỏ do xung đột băm (Hash Collision) hoặc giải phóng lặp giữa các liên kết phối ngẫu.</t>
+        </is>
+      </c>
+      <c r="K13" s="18" t="inlineStr">
         <is>
           <t>Sinh nhiều member_id có cùng giá trị modulo 64 (ví dụ: id=1 và id=65) kết hợp xen kẽ các lệnh tạo, xóa và dọn dẹp bộ nhớ.</t>
         </is>
@@ -1297,7 +1376,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>raw_data_size (size_t)</t>
+          <t>data buffer, declared_len</t>
         </is>
       </c>
       <c r="F14" s="21" t="inlineStr">
@@ -1307,7 +1386,7 @@
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>CWE-131 / CWE-125</t>
+          <t>CWE-131 / CWE-125 (CVE-2020-0796)</t>
         </is>
       </c>
       <c r="H14" s="22" t="inlineStr">
@@ -1317,12 +1396,17 @@
       </c>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>Xử lý sai kích thước dữ liệu đầu vào khi size &lt; sizeof(Header) hoặc size cực lớn gần bằng SIZE_MAX, dẫn đến ép kiểu con trỏ không hợp lệ và đọc ngoài biên bộ nhớ.</t>
+          <t>Nhánh size &lt; sizeof(uint16_t); nhánh declared_len &gt; 0 và vòng lặp đọc checksum theo declared_len</t>
         </is>
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>Cung cấp size = 0, size = 1, size = sizeof(FuzzMemberPayload) - 1, size = 0xFFFFFFFF.</t>
+          <t>Xử lý sai kích thước dữ liệu đầu vào khi size &lt; sizeof(Header) hoặc declared_len &gt; size thực tế, dẫn đến ép kiểu con trỏ không hợp lệ và đọc ngoài biên bộ nhớ (OOB Read).</t>
+        </is>
+      </c>
+      <c r="K14" s="13" t="inlineStr">
+        <is>
+          <t>Cung cấp size = 0, size = 1, size = sizeof(FuzzMemberPayload) - 1, size = 0xFFFFFFFF; byte đầu tiên chứa declared_len cực đại.</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1426,7 @@
       </c>
       <c r="E15" s="18" t="inlineStr">
         <is>
-          <t>node-&gt;spouse pointer</t>
+          <t>node1-&gt;spouse, node2-&gt;spouse</t>
         </is>
       </c>
       <c r="F15" s="20" t="inlineStr">
@@ -1352,7 +1436,7 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>CWE-476 / CWE-401</t>
+          <t>CWE-476 / CWE-401 (CVE-2020-14386)</t>
         </is>
       </c>
       <c r="H15" s="22" t="inlineStr">
@@ -1362,12 +1446,17 @@
       </c>
       <c r="I15" s="18" t="inlineStr">
         <is>
-          <t>Giải tham chiếu con trỏ NULL khi truy cập thông tin phối ngẫu mà không kiểm tra tính hợp lệ; hoặc rò rỉ bộ nhớ khi gán đè con trỏ phối ngẫu mà không giải phóng nút cũ.</t>
+          <t>Nhánh node1 != NULL kết hợp nhánh node2 == NULL; nhánh gán đè liên kết phối ngẫu nhiều lần</t>
         </is>
       </c>
       <c r="J15" s="18" t="inlineStr">
         <is>
-          <t>Gửi spouse_id = 0 kết hợp opcode cập nhật liên kết phối ngẫu nhiều lần liên tiếp trên cùng một node.</t>
+          <t>Giải tham chiếu con trỏ NULL khi truy cập thông tin phối ngẫu mà không kiểm tra tính hợp lệ; hoặc rò rỉ bộ nhớ (Memory Leak) khi gán đè con trỏ phối ngẫu mà không giải phóng nút cũ.</t>
+        </is>
+      </c>
+      <c r="K15" s="18" t="inlineStr">
+        <is>
+          <t>Gửi spouse_id = 0 (khiến node2 = NULL) kết hợp opcode=3 cập nhật liên kết phối ngẫu nhiều lần liên tiếp trên cùng một node.</t>
         </is>
       </c>
     </row>
@@ -1382,24 +1471,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C9"/>
+  <dimension ref="B2:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="85" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>HƯỚNG DẪN THỰC THI KIỂM THỬ ĐỘNG (LIBFUZZER &amp; AFL++)</t>
+          <t>HƯỚNG DẪN THỰC THI KIỂM THỬ ĐỘNG &amp; THU THẬP ĐỘ PHỦ (CODE COVERAGE)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Tài liệu hướng dẫn biên dịch mã nguồn C mô phỏng cùng các sanitizers</t>
+          <t>Tài liệu hướng dẫn biên dịch mã nguồn C mô phỏng cùng Sanitizers và đo Code Coverage bằng LLVM Cov</t>
         </is>
       </c>
     </row>
@@ -1412,63 +1501,79 @@
       <c r="C5" s="23" t="inlineStr">
         <is>
           <t>Cài đặt LLVM Clang phiên bản 16+ hoặc AFL++ trên Linux/WSL2:
-  sudo apt install clang llvm libfuzzer-dev afl++</t>
+  sudo apt update &amp;&amp; sudo apt install -y clang llvm libfuzzer-dev afl++</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Bước 2: Biên dịch với libFuzzer + ASan + UBSan</t>
+          <t>Bước 2: Biên dịch Fuzzer với Clang + ASan + UBSan</t>
         </is>
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>Lệnh biên dịch trực tiếp harness:
-  clang -fsanitize=fuzzer,address,undefined -g -O1 clan_genealogy_fuzzer.c -o fuzzer_clan</t>
+          <t>Biên dịch harness đa bước kiểm thử an toàn bộ nhớ:
+  clang -fsanitize=fuzzer,address,undefined -DLIBFUZZER_RUN -g -O1 clan_genealogy_fuzzer.c -o fuzzer_clan</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Bước 3: Khởi chạy Fuzzing với libFuzzer</t>
+          <t>Bước 3: Khởi chạy Fuzzing tìm lỗi</t>
         </is>
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>Tạo thư mục corpus và bắt đầu fuzzing với giới hạn độ dài payload:
-  mkdir corpus
-  ./fuzzer_clan corpus/ -max_len=512 -timeout=5 -runs=10000000</t>
+          <t>Tạo thư mục corpus và bắt đầu fuzzing với giới hạn độ dài payload đa bước:
+  mkdir -p corpus
+  ./fuzzer_clan corpus/ -max_len=1024 -timeout=5 -runs=10000000</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Bước 4: Biên dịch và chạy với AFL++</t>
+          <t>Bước 4: Thu thập độ phủ mã nguồn (Source-based Code Coverage)</t>
         </is>
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Biên dịch với afl-clang-fast:
-  afl-clang-fast -fsanitize=address -g clan_genealogy_fuzzer.c -o fuzzer_afl
-  afl-fuzz -i corpus/ -o findings/ -m none -- ./fuzzer_afl</t>
+          <t>Biên dịch với cờ sinh profile coverage của Clang:
+  clang -fprofile-instr-generate -fcoverage-mapping -g clan_genealogy_fuzzer.c -o fuzzer_cov
+  LLVM_PROFILE_FILE="clan_%p.profraw" ./fuzzer_cov
+  llvm-profdata merge -sparse clan_*.profraw -o clan.profdata
+  llvm-cov report ./fuzzer_cov -instr-profile=clan.profdata
+  llvm-cov show ./fuzzer_cov -instr-profile=clan.profdata -format=html -output-dir=coverage_report</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Bước 5: Phân tích Crash &amp; Báo cáo Lỗi</t>
+          <t>Bước 5: Chạy độc lập trên Windows bằng GCC (Không cần Clang)</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Khi ASan bắt được crash (Heap-buffer-overflow, UAF, Stack-overflow):
-  1. File crash được lưu dạng crash-xxxx hoặc findings/default/crashes/
-  2. Chạy tái hiện: ./fuzzer_clan crash-xxxx
-  3. Đọc địa chỉ con trỏ và stack trace để định vị dòng code lỗi.</t>
+          <t>Biên dịch và chạy trực tiếp standalone multi-step fuzzer:
+  gcc -Wall -Wextra clan_genealogy_fuzzer.c -o fuzzer_clan.exe
+  .\fuzzer_clan.exe</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Bước 6: Tái hiện lỗi từ file Crash (Reproduce Bug)</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>Khi phát hiện crash (crash-xxxx hoặc crash_payload.bin), chạy kiểm chứng:
+  ./fuzzer_clan crash-xxxx
+  .\fuzzer_clan.exe crash_payload.bin</t>
         </is>
       </c>
     </row>

</xml_diff>